<commit_message>
FILTERXML y WEBSERVICE + ruta /fetch en el host
- FILTERXML(xml, xpath): XPath local con DOMParser (Univer traía el nombre
  pero no el cálculo → daba #NAME?).
- WEBSERVICE(url): trae texto de una URL vía el host C#. El motor de Univer
  no admite funciones async (una Promise se interpreta como matriz → #SPILL!),
  así que usa caché síncrona + refresco por reescritura de la fórmula.
- Server.cs: ruta GET /fetch?url= con HttpClient (timeout, límite 256KB,
  solo http/https) para sortear el CSP de WebView2.
- Libro de ejemplos: sección Web/XML en el banco; cubo y async documentados
  en Limitaciones.
- README: tablas Web/XML y nota de que ingeniería/estadística son nativas.

Verificado en la app: FILTERXML=7, ENCODEURL ok, WEBSERVICE trae datos reales.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ejemplos/Ejemplos XlsView.xlsx
+++ b/ejemplos/Ejemplos XlsView.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="306">
   <si>
     <t>📊 XlsView — Ejemplos de fórmulas, funciones y macros</t>
   </si>
@@ -786,6 +786,27 @@
   </si>
   <si>
     <t>=TRIMESTRE(DATE(2026,8,1))</t>
+  </si>
+  <si>
+    <t>Web / XML</t>
+  </si>
+  <si>
+    <t>ENCODEURL — codifica una URL</t>
+  </si>
+  <si>
+    <t>=ENCODEURL("a b&amp;c")</t>
+  </si>
+  <si>
+    <t>FILTERXML — XPath sobre XML</t>
+  </si>
+  <si>
+    <t>=FILTERXML("&lt;r&gt;&lt;i&gt;7&lt;/i&gt;&lt;/r&gt;","//i")</t>
+  </si>
+  <si>
+    <t>WEBSERVICE — texto de una URL</t>
+  </si>
+  <si>
+    <t>=WEBSERVICE("https://api.github.com/zen")</t>
   </si>
   <si>
     <t>⚡ Macros — automatización con JavaScript</t>
@@ -922,6 +943,21 @@
   </si>
   <si>
     <t>Envolver en SUM/MAX: SÍ funciona =SUM(MAP(...))</t>
+  </si>
+  <si>
+    <t>CUBEMEMBER, CUBEVALUE…</t>
+  </si>
+  <si>
+    <t>#NAME? (sin OLAP)</t>
+  </si>
+  <si>
+    <t>Las 7 funciones de cubo necesitan un servidor OLAP; no aplican sin backend</t>
+  </si>
+  <si>
+    <t>Funciones async (Promise)</t>
+  </si>
+  <si>
+    <t>El motor no admite async; para red usar WEBSERVICE (caché síncrona del host)</t>
   </si>
   <si>
     <t>✔ MAP y REDUCE SÍ funcionan si su array se consume dentro de una función:</t>
@@ -2730,7 +2766,7 @@
   <sheetPr>
     <tabColor rgb="FF9E480E"/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3267,8 +3303,50 @@
         <f>TRIMESTRE(DATE(2026,8,1))</f>
       </c>
     </row>
+    <row r="49" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="D50" s="12">
+        <f>ENCODEURL("a b&amp;c")</f>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C51" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="D51" s="12">
+        <f>FILTERXML("&lt;r&gt;&lt;i&gt;7&lt;/i&gt;&lt;/r&gt;","//i")</f>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="4"/>
+      <c r="B52" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="D52" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A5:D5"/>
@@ -3278,6 +3356,7 @@
     <mergeCell ref="A36:D36"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A49:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3299,21 +3378,21 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -3321,64 +3400,64 @@
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="16" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" ht="112" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="16" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" ht="98" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="16" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" ht="56" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="16" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" ht="112" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="16" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" ht="126" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="16" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -3397,7 +3476,7 @@
   <sheetPr>
     <tabColor rgb="FFED7D31"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3407,7 +3486,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3415,7 +3494,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3424,103 +3503,127 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="18" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="21" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="18" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="21" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="18" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D9" s="20" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="C11" s="19" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="24" t="s">
-        <v>290</v>
-      </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="25" t="s">
-        <v>291</v>
-      </c>
-      <c r="C12" s="26">
-        <f>SUM(MAP({2,4,6},LAMBDA(v,v*v)))</f>
-      </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="25" t="s">
-        <v>292</v>
-      </c>
-      <c r="C13" s="26">
-        <f>REDUCE(0,{1,2,3,4,5},LAMBDA(a,v,a+v))</f>
-      </c>
+      <c r="D11" s="20" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>293</v>
+        <v>303</v>
       </c>
       <c r="C14" s="26">
+        <f>SUM(MAP({2,4,6},LAMBDA(v,v*v)))</f>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="C15" s="26">
+        <f>REDUCE(0,{1,2,3,4,5},LAMBDA(a,v,a+v))</f>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="C16" s="26">
         <f>SUM({1,2,3,4,5})</f>
       </c>
     </row>
@@ -3528,7 +3631,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B13:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
chore: actualizar libro de ejemplo
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ejemplos/Ejemplos XlsView.xlsx
+++ b/ejemplos/Ejemplos XlsView.xlsx
@@ -992,7 +992,7 @@
         <v>IF anidado (if/then/else)</v>
       </c>
     </row>
-    <row r="6" ht="20.25" customHeight="1">
+    <row r="6" ht="16.5" customHeight="1">
       <c s="12" r="B6" t="str">
         <v>IF simple</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>tres</v>
       </c>
     </row>
-    <row r="10" ht="20.25" customHeight="1">
+    <row r="10" ht="16.5" customHeight="1">
       <c s="12" r="B10" t="str">
         <v>IFERROR envuelve un error</v>
       </c>
@@ -1048,8 +1048,8 @@
         <v>=IFERROR(10/0,"sin dividir")</v>
       </c>
       <c s="14" r="D10" t="str">
-        <f>IFERROR(10/0,"sin dividir")</f>
-        <v>sin dividir</v>
+        <f>IFERROR(10/0,"division por cero")</f>
+        <v>division por cero</v>
       </c>
     </row>
     <row r="11" ht="20.25" customHeight="1">
@@ -1225,7 +1225,7 @@
         <v>Lógicas</v>
       </c>
     </row>
-    <row r="6" ht="20.25" customHeight="1">
+    <row r="6" ht="16.5" customHeight="1">
       <c s="12" r="B6" t="str">
         <v>AND / OR / NOT</v>
       </c>

</xml_diff>